<commit_message>
Update to corrected dataset, analyses 1-7, and external validation
- De-identified data corrected to true patient grouping (194 patients, 8
  bilateral; previously mis-grouped by initials). External validation cohort
  (54 independent eyes) added.
- Pipeline reproduces from de-identified data/processed/*.csv (the
  name-containing sources are withheld); analyses 1-7 including the ablations
  and the non-negative formula refit with external validation.
- Link the de-identified Hugging Face dataset; rewrite README; remove the
  stale initials spreadsheet. No patient names anywhere in code or data.
</commit_message>
<xml_diff>
--- a/experiments/outputs/tables/table04_mixed_effects.xlsx
+++ b/experiments/outputs/tables/table04_mixed_effects.xlsx
@@ -495,13 +495,13 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>-0.1448663800913659</v>
+        <v>-0.1391250587657216</v>
       </c>
       <c r="D2">
-        <v>0.1102035457156001</v>
+        <v>0.11057849678558</v>
       </c>
       <c r="E2">
-        <v>0.1886663433822834</v>
+        <v>0.2083351493319586</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -510,13 +510,13 @@
         <v>9</v>
       </c>
       <c r="C3">
-        <v>-0.9310031931600329</v>
+        <v>-0.9589498619096763</v>
       </c>
       <c r="D3">
-        <v>1.523251177479574</v>
+        <v>1.51955059554671</v>
       </c>
       <c r="E3">
-        <v>0.5410706279449553</v>
+        <v>0.5279917146998854</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -525,13 +525,13 @@
         <v>10</v>
       </c>
       <c r="C4">
-        <v>-0.05129290422928121</v>
+        <v>-0.048493725841565</v>
       </c>
       <c r="D4">
-        <v>0.05578257418639684</v>
+        <v>0.05657564589197732</v>
       </c>
       <c r="E4">
-        <v>0.3578263522733045</v>
+        <v>0.3913628608683953</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -540,13 +540,13 @@
         <v>11</v>
       </c>
       <c r="C5">
-        <v>0.05036525265151422</v>
+        <v>0.1416370876219361</v>
       </c>
       <c r="D5">
-        <v>0.9491055547986338</v>
+        <v>0.9521759578796295</v>
       </c>
       <c r="E5">
-        <v>0.9576793068288424</v>
+        <v>0.8817501484171588</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -555,13 +555,13 @@
         <v>12</v>
       </c>
       <c r="C6">
-        <v>-0.01357220233521698</v>
+        <v>-0.02205367914474993</v>
       </c>
       <c r="D6">
-        <v>0.1044700117765192</v>
+        <v>0.1046277567742407</v>
       </c>
       <c r="E6">
-        <v>0.8966338223294239</v>
+        <v>0.8330571513430733</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -570,13 +570,13 @@
         <v>13</v>
       </c>
       <c r="C7">
-        <v>0.008749870821289</v>
+        <v>0.004908063224165095</v>
       </c>
       <c r="D7">
-        <v>0.03150388570155799</v>
+        <v>0.03127806664074544</v>
       </c>
       <c r="E7">
-        <v>0.7812124007915713</v>
+        <v>0.8753101901844864</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -585,13 +585,13 @@
         <v>14</v>
       </c>
       <c r="C8">
-        <v>0.4818939444254197</v>
+        <v>0.4609842960544077</v>
       </c>
       <c r="D8">
-        <v>0.3024740237011747</v>
+        <v>0.3036522182477235</v>
       </c>
       <c r="E8">
-        <v>0.1111210182226772</v>
+        <v>0.1289810038594135</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -600,13 +600,13 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>0.002467014010879173</v>
+        <v>0.00230446008104804</v>
       </c>
       <c r="D9">
-        <v>0.01205653418060679</v>
+        <v>0.01200883839427776</v>
       </c>
       <c r="E9">
-        <v>0.837868640281761</v>
+        <v>0.8478228861415131</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -615,13 +615,13 @@
         <v>16</v>
       </c>
       <c r="C10">
-        <v>-0.009280553963028489</v>
+        <v>-0.008762628722446887</v>
       </c>
       <c r="D10">
-        <v>0.01282498030330078</v>
+        <v>0.01281602269920323</v>
       </c>
       <c r="E10">
-        <v>0.4692922736696651</v>
+        <v>0.4941491491320252</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -630,13 +630,13 @@
         <v>17</v>
       </c>
       <c r="C11">
-        <v>0.001203326238297283</v>
+        <v>0.001123564418633659</v>
       </c>
       <c r="D11">
-        <v>0.001043602871246725</v>
+        <v>0.001052044401362093</v>
       </c>
       <c r="E11">
-        <v>0.2488898830900254</v>
+        <v>0.2855286593381592</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -645,13 +645,13 @@
         <v>18</v>
       </c>
       <c r="C12">
-        <v>0.003821883859841386</v>
+        <v>0.00361944019881766</v>
       </c>
       <c r="D12">
-        <v>0.001998087546831712</v>
+        <v>0.001980768402464649</v>
       </c>
       <c r="E12">
-        <v>0.05577737878474221</v>
+        <v>0.06765603348061346</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -660,13 +660,13 @@
         <v>19</v>
       </c>
       <c r="C13">
-        <v>2.577758327525748E-05</v>
+        <v>-8.514994418098264E-06</v>
       </c>
       <c r="D13">
-        <v>0.0002213326519734396</v>
+        <v>0.0002199318144337138</v>
       </c>
       <c r="E13">
-        <v>0.9072837512575187</v>
+        <v>0.9691164024973525</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -675,13 +675,13 @@
         <v>20</v>
       </c>
       <c r="C14">
-        <v>-0.09019641470447093</v>
+        <v>-0.0838760942550504</v>
       </c>
       <c r="D14">
-        <v>0.08630570097226382</v>
+        <v>0.08600593884775123</v>
       </c>
       <c r="E14">
-        <v>0.2959857144138873</v>
+        <v>0.3294431712440361</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -690,13 +690,13 @@
         <v>21</v>
       </c>
       <c r="C15">
-        <v>-0.05585026034979799</v>
+        <v>-0.04904164180141282</v>
       </c>
       <c r="D15">
-        <v>0.03288461486961308</v>
+        <v>0.03240330894614876</v>
       </c>
       <c r="E15">
-        <v>0.08943785308769039</v>
+        <v>0.130158703699626</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -705,13 +705,13 @@
         <v>22</v>
       </c>
       <c r="C16">
-        <v>-0.01168391812163783</v>
+        <v>-0.01648759373261817</v>
       </c>
       <c r="D16">
-        <v>0.3193371948246191</v>
+        <v>0.3205686587270434</v>
       </c>
       <c r="E16">
-        <v>0.9708134896717259</v>
+        <v>0.9589810215279451</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -720,13 +720,13 @@
         <v>23</v>
       </c>
       <c r="C17">
-        <v>0.1852874848011764</v>
+        <v>0.1727483067157566</v>
       </c>
       <c r="D17">
-        <v>0.134170637227228</v>
+        <v>0.1332885219446641</v>
       </c>
       <c r="E17">
-        <v>0.16728392261139</v>
+        <v>0.1949589886341956</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -735,13 +735,13 @@
         <v>24</v>
       </c>
       <c r="C18">
-        <v>0.1074807879844152</v>
+        <v>0.09012685925370531</v>
       </c>
       <c r="D18">
-        <v>0.07149995673843905</v>
+        <v>0.07113736888888954</v>
       </c>
       <c r="E18">
-        <v>0.132780075548437</v>
+        <v>0.2051763369140387</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -750,13 +750,13 @@
         <v>25</v>
       </c>
       <c r="C19">
-        <v>-0.0001171264723015678</v>
+        <v>-0.0002033028938761196</v>
       </c>
       <c r="D19">
-        <v>0.0006814901748288186</v>
+        <v>0.0006874662564016871</v>
       </c>
       <c r="E19">
-        <v>0.8635411672932402</v>
+        <v>0.7674379534958721</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -765,13 +765,13 @@
         <v>26</v>
       </c>
       <c r="C20">
-        <v>0.02863857771017079</v>
+        <v>0.02763614064057999</v>
       </c>
       <c r="D20">
-        <v>0.0231487980156922</v>
+        <v>0.02337388637894608</v>
       </c>
       <c r="E20">
-        <v>0.216030722702533</v>
+        <v>0.2370664112622287</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -780,13 +780,13 @@
         <v>27</v>
       </c>
       <c r="C21">
-        <v>-0.03308007735437417</v>
+        <v>-0.04871412512018575</v>
       </c>
       <c r="D21">
-        <v>0.06658772239678983</v>
+        <v>0.06723077548876509</v>
       </c>
       <c r="E21">
-        <v>0.6193375423769303</v>
+        <v>0.468709277505119</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -795,13 +795,13 @@
         <v>28</v>
       </c>
       <c r="C22">
-        <v>0.01047938777845519</v>
+        <v>0.01022576656941238</v>
       </c>
       <c r="D22">
-        <v>0.003618546596878251</v>
+        <v>0.003598529229173258</v>
       </c>
       <c r="E22">
-        <v>0.003779268276631196</v>
+        <v>0.004488049923004502</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -810,13 +810,13 @@
         <v>29</v>
       </c>
       <c r="C23">
-        <v>0.09421857825286843</v>
+        <v>0.09521333269208238</v>
       </c>
       <c r="D23">
-        <v>0.06535700522790819</v>
+        <v>0.06520665468166327</v>
       </c>
       <c r="E23">
-        <v>0.1494155960494466</v>
+        <v>0.1442411175584216</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -827,13 +827,13 @@
         <v>8</v>
       </c>
       <c r="C24">
-        <v>-0.01522652797060608</v>
+        <v>-0.01522652777432152</v>
       </c>
       <c r="D24">
-        <v>0.1341517637427899</v>
+        <v>0.1330362364377713</v>
       </c>
       <c r="E24">
-        <v>0.9096323737879143</v>
+        <v>0.9088779190989136</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -842,13 +842,13 @@
         <v>9</v>
       </c>
       <c r="C25">
-        <v>-0.6429686072431945</v>
+        <v>-0.6429686056204736</v>
       </c>
       <c r="D25">
-        <v>1.801409220104907</v>
+        <v>1.809990247124794</v>
       </c>
       <c r="E25">
-        <v>0.721147695201691</v>
+        <v>0.7224149035914631</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -857,13 +857,13 @@
         <v>10</v>
       </c>
       <c r="C26">
-        <v>-0.1071684836868455</v>
+        <v>-0.1071684829959763</v>
       </c>
       <c r="D26">
-        <v>0.06902029115281012</v>
+        <v>0.06727747430062077</v>
       </c>
       <c r="E26">
-        <v>0.1204924758029825</v>
+        <v>0.1111753088967947</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -872,13 +872,13 @@
         <v>11</v>
       </c>
       <c r="C27">
-        <v>-1.864280144546278</v>
+        <v>-1.86428014935259</v>
       </c>
       <c r="D27">
-        <v>1.121818680792101</v>
+        <v>1.119621876751543</v>
       </c>
       <c r="E27">
-        <v>0.09654539811235902</v>
+        <v>0.09589320540327669</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -887,13 +887,13 @@
         <v>12</v>
       </c>
       <c r="C28">
-        <v>0.04797132758352607</v>
+        <v>0.04797132756217869</v>
       </c>
       <c r="D28">
-        <v>0.1227825274088899</v>
+        <v>0.1223649512155423</v>
       </c>
       <c r="E28">
-        <v>0.6960178300675988</v>
+        <v>0.6950324504133131</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -902,13 +902,13 @@
         <v>13</v>
       </c>
       <c r="C29">
-        <v>-0.05407809847310788</v>
+        <v>-0.05407809856808731</v>
       </c>
       <c r="D29">
-        <v>0.03706319336755664</v>
+        <v>0.03687896642121283</v>
       </c>
       <c r="E29">
-        <v>0.144543578095449</v>
+        <v>0.1425483373239978</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -917,13 +917,13 @@
         <v>14</v>
       </c>
       <c r="C30">
-        <v>0.4971505738981057</v>
+        <v>0.4971505738850149</v>
       </c>
       <c r="D30">
-        <v>0.3587475873032649</v>
+        <v>0.3594881332713202</v>
       </c>
       <c r="E30">
-        <v>0.1658095426642777</v>
+        <v>0.1666832172487347</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -932,13 +932,13 @@
         <v>15</v>
       </c>
       <c r="C31">
-        <v>-0.007793181201334687</v>
+        <v>-0.007793181200902091</v>
       </c>
       <c r="D31">
-        <v>0.01414679773444198</v>
+        <v>0.01414600566328136</v>
       </c>
       <c r="E31">
-        <v>0.5817162648731155</v>
+        <v>0.5816951189985727</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -947,13 +947,13 @@
         <v>16</v>
       </c>
       <c r="C32">
-        <v>-0.008669519524899054</v>
+        <v>-0.008669519524494549</v>
       </c>
       <c r="D32">
-        <v>0.01513937190749122</v>
+        <v>0.01512142048769461</v>
       </c>
       <c r="E32">
-        <v>0.5668835678347759</v>
+        <v>0.5664232679306331</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -962,13 +962,13 @@
         <v>17</v>
       </c>
       <c r="C33">
-        <v>0.0001865776249381574</v>
+        <v>0.0001865776246262631</v>
       </c>
       <c r="D33">
-        <v>0.001243446711192246</v>
+        <v>0.001240924959117651</v>
       </c>
       <c r="E33">
-        <v>0.8807261535180956</v>
+        <v>0.8804855898585394</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -977,13 +977,13 @@
         <v>18</v>
       </c>
       <c r="C34">
-        <v>-0.0006409746581465593</v>
+        <v>-0.000640974659216334</v>
       </c>
       <c r="D34">
-        <v>0.002379962662763442</v>
+        <v>0.002388743833108421</v>
       </c>
       <c r="E34">
-        <v>0.7876824360832896</v>
+        <v>0.7884443408370452</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -992,13 +992,13 @@
         <v>19</v>
       </c>
       <c r="C35">
-        <v>1.36881524665082E-06</v>
+        <v>1.368815294873868E-06</v>
       </c>
       <c r="D35">
-        <v>0.0002608142315679239</v>
+        <v>0.0002603270219501484</v>
       </c>
       <c r="E35">
-        <v>0.9958125308898151</v>
+        <v>0.9958046938435449</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -1007,13 +1007,13 @@
         <v>20</v>
       </c>
       <c r="C36">
-        <v>-0.1057550727604133</v>
+        <v>-0.105755072683866</v>
       </c>
       <c r="D36">
-        <v>0.1007246794109528</v>
+        <v>0.101767353364095</v>
       </c>
       <c r="E36">
-        <v>0.29374477345422</v>
+        <v>0.2987188625300325</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -1022,13 +1022,13 @@
         <v>21</v>
       </c>
       <c r="C37">
-        <v>-0.01013787685069185</v>
+        <v>-0.01013787701316518</v>
       </c>
       <c r="D37">
-        <v>0.03875382610717019</v>
+        <v>0.03919607299803562</v>
       </c>
       <c r="E37">
-        <v>0.7936323122907006</v>
+        <v>0.7959089878196828</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -1037,13 +1037,13 @@
         <v>22</v>
       </c>
       <c r="C38">
-        <v>0.2474855315794836</v>
+        <v>0.2474855315578516</v>
       </c>
       <c r="D38">
-        <v>0.3795665967147624</v>
+        <v>0.3795275911076649</v>
       </c>
       <c r="E38">
-        <v>0.5143873880041923</v>
+        <v>0.5143441605649415</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -1052,13 +1052,13 @@
         <v>23</v>
       </c>
       <c r="C39">
-        <v>-0.02418527920031763</v>
+        <v>-0.02418527919313794</v>
       </c>
       <c r="D39">
-        <v>0.1580642554364013</v>
+        <v>0.1579234700474763</v>
       </c>
       <c r="E39">
-        <v>0.8783910504708656</v>
+        <v>0.8782834832577497</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -1067,13 +1067,13 @@
         <v>24</v>
       </c>
       <c r="C40">
-        <v>0.01708553384495523</v>
+        <v>0.01708553385434895</v>
       </c>
       <c r="D40">
-        <v>0.08498134941073311</v>
+        <v>0.08484787024144307</v>
       </c>
       <c r="E40">
-        <v>0.8406591691752311</v>
+        <v>0.8404118678108081</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -1082,13 +1082,13 @@
         <v>25</v>
       </c>
       <c r="C41">
-        <v>0.0002285931789694578</v>
+        <v>0.0002285931796511204</v>
       </c>
       <c r="D41">
-        <v>0.0008210490517724785</v>
+        <v>0.0008215558757867585</v>
       </c>
       <c r="E41">
-        <v>0.7806930515783224</v>
+        <v>0.7808248864554681</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -1097,13 +1097,13 @@
         <v>26</v>
       </c>
       <c r="C42">
-        <v>0.05575421933567465</v>
+        <v>0.05575421932085235</v>
       </c>
       <c r="D42">
-        <v>0.02711250747162261</v>
+        <v>0.02710921198694439</v>
       </c>
       <c r="E42">
-        <v>0.03974376682600823</v>
+        <v>0.03971969728097039</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -1112,13 +1112,13 @@
         <v>27</v>
       </c>
       <c r="C43">
-        <v>0.09595946940223249</v>
+        <v>0.09595946891881103</v>
       </c>
       <c r="D43">
-        <v>0.08188674872691147</v>
+        <v>0.08023741085241413</v>
       </c>
       <c r="E43">
-        <v>0.2412549162318056</v>
+        <v>0.2317183215034622</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -1127,13 +1127,13 @@
         <v>28</v>
       </c>
       <c r="C44">
-        <v>0.0008296155115566836</v>
+        <v>0.000829615512243329</v>
       </c>
       <c r="D44">
-        <v>0.0042791564679505</v>
+        <v>0.004304476465330409</v>
       </c>
       <c r="E44">
-        <v>0.8462748479125903</v>
+        <v>0.8471679231034944</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -1142,13 +1142,13 @@
         <v>29</v>
       </c>
       <c r="C45">
-        <v>0.3262999474371036</v>
+        <v>0.3262999476705063</v>
       </c>
       <c r="D45">
-        <v>0.07534397742956626</v>
+        <v>0.07537066875624841</v>
       </c>
       <c r="E45">
-        <v>1.485663410336829E-05</v>
+        <v>1.49604671727498E-05</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -1159,13 +1159,13 @@
         <v>8</v>
       </c>
       <c r="C46">
-        <v>0.1951503797961407</v>
+        <v>0.1936462343521487</v>
       </c>
       <c r="D46">
-        <v>0.1271395977566463</v>
+        <v>0.1274431521723111</v>
       </c>
       <c r="E46">
-        <v>0.1248010292678061</v>
+        <v>0.1286438629208462</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -1174,13 +1174,13 @@
         <v>9</v>
       </c>
       <c r="C47">
-        <v>-3.277516223244545</v>
+        <v>-3.465489900651035</v>
       </c>
       <c r="D47">
-        <v>1.741546016369544</v>
+        <v>1.777031245901563</v>
       </c>
       <c r="E47">
-        <v>0.05984173672246138</v>
+        <v>0.05115741069608033</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -1189,13 +1189,13 @@
         <v>10</v>
       </c>
       <c r="C48">
-        <v>-0.01348066628066549</v>
+        <v>-0.004093628962377588</v>
       </c>
       <c r="D48">
-        <v>0.0649095428013738</v>
+        <v>0.06588656654055529</v>
       </c>
       <c r="E48">
-        <v>0.8354757981330982</v>
+        <v>0.9504581392307416</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -1204,13 +1204,13 @@
         <v>11</v>
       </c>
       <c r="C49">
-        <v>0.1584493157669628</v>
+        <v>0.3198110959908957</v>
       </c>
       <c r="D49">
-        <v>1.100411531475193</v>
+        <v>1.102882416372764</v>
       </c>
       <c r="E49">
-        <v>0.8855076060004209</v>
+        <v>0.7718334438100042</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -1219,13 +1219,13 @@
         <v>12</v>
       </c>
       <c r="C50">
-        <v>-0.06473469717197657</v>
+        <v>-0.08622365384019845</v>
       </c>
       <c r="D50">
-        <v>0.1216374095676745</v>
+        <v>0.1207585511886872</v>
       </c>
       <c r="E50">
-        <v>0.5945916516577585</v>
+        <v>0.4752166910242109</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -1234,13 +1234,13 @@
         <v>13</v>
       </c>
       <c r="C51">
-        <v>0.03535170526361804</v>
+        <v>0.02784941073551905</v>
       </c>
       <c r="D51">
-        <v>0.03635345426808167</v>
+        <v>0.0364851454225628</v>
       </c>
       <c r="E51">
-        <v>0.3308296186814146</v>
+        <v>0.4452796119837386</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -1249,13 +1249,13 @@
         <v>14</v>
       </c>
       <c r="C52">
-        <v>-0.06255295217072963</v>
+        <v>-0.105027053861575</v>
       </c>
       <c r="D52">
-        <v>0.3539944089148792</v>
+        <v>0.3529098743528737</v>
       </c>
       <c r="E52">
-        <v>0.8597392918915667</v>
+        <v>0.7660061488652543</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -1264,13 +1264,13 @@
         <v>15</v>
       </c>
       <c r="C53">
-        <v>0.0129174478843011</v>
+        <v>0.01330691866081654</v>
       </c>
       <c r="D53">
-        <v>0.01389212933012684</v>
+        <v>0.01386002316382789</v>
       </c>
       <c r="E53">
-        <v>0.3524542922144256</v>
+        <v>0.3370081409862896</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -1279,13 +1279,13 @@
         <v>16</v>
       </c>
       <c r="C54">
-        <v>0.004349093822877492</v>
+        <v>0.005406764652837417</v>
       </c>
       <c r="D54">
-        <v>0.01486143277337019</v>
+        <v>0.01483716872792426</v>
       </c>
       <c r="E54">
-        <v>0.7697950656824104</v>
+        <v>0.7155542847797105</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -1294,13 +1294,13 @@
         <v>17</v>
       </c>
       <c r="C55">
-        <v>0.000964976019328157</v>
+        <v>0.0008664923464290091</v>
       </c>
       <c r="D55">
-        <v>0.001211323155329936</v>
+        <v>0.001219097130560948</v>
       </c>
       <c r="E55">
-        <v>0.4256661147873236</v>
+        <v>0.4772294790855427</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -1309,13 +1309,13 @@
         <v>18</v>
       </c>
       <c r="C56">
-        <v>0.003841978551857693</v>
+        <v>0.00373049361367373</v>
       </c>
       <c r="D56">
-        <v>0.002301772137445069</v>
+        <v>0.002298987275634551</v>
       </c>
       <c r="E56">
-        <v>0.09508975760266089</v>
+        <v>0.1046603463185799</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -1324,13 +1324,13 @@
         <v>19</v>
       </c>
       <c r="C57">
-        <v>0.0003717871086292294</v>
+        <v>0.0003407657797036075</v>
       </c>
       <c r="D57">
-        <v>0.0002525459124986323</v>
+        <v>0.0002534318588554263</v>
       </c>
       <c r="E57">
-        <v>0.1409786189724105</v>
+        <v>0.1787527830423645</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -1339,13 +1339,13 @@
         <v>20</v>
       </c>
       <c r="C58">
-        <v>-0.2040692910685077</v>
+        <v>-0.1995195340818603</v>
       </c>
       <c r="D58">
-        <v>0.09820226626087333</v>
+        <v>0.0980799042622027</v>
       </c>
       <c r="E58">
-        <v>0.03770468696099086</v>
+        <v>0.0419258933607103</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -1354,13 +1354,13 @@
         <v>21</v>
       </c>
       <c r="C59">
-        <v>-0.08902722096974593</v>
+        <v>-0.0795494744238316</v>
       </c>
       <c r="D59">
-        <v>0.03725665824748503</v>
+        <v>0.03702735075996743</v>
       </c>
       <c r="E59">
-        <v>0.01686832091766432</v>
+        <v>0.03168217703654997</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -1369,13 +1369,13 @@
         <v>22</v>
       </c>
       <c r="C60">
-        <v>-0.2593808815387729</v>
+        <v>-0.2615286422307555</v>
       </c>
       <c r="D60">
-        <v>0.3690493607961591</v>
+        <v>0.3709519820001154</v>
       </c>
       <c r="E60">
-        <v>0.4821584575609351</v>
+        <v>0.4807976625901825</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -1384,13 +1384,13 @@
         <v>23</v>
       </c>
       <c r="C61">
-        <v>0.3291983924338194</v>
+        <v>0.3194307594705948</v>
       </c>
       <c r="D61">
-        <v>0.1541543070786401</v>
+        <v>0.1531404878163821</v>
       </c>
       <c r="E61">
-        <v>0.03271920055774818</v>
+        <v>0.03699063110216985</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -1399,13 +1399,13 @@
         <v>24</v>
       </c>
       <c r="C62">
-        <v>0.1666786863322892</v>
+        <v>0.1520635675826608</v>
       </c>
       <c r="D62">
-        <v>0.08101368698802103</v>
+        <v>0.08183676289058923</v>
       </c>
       <c r="E62">
-        <v>0.03964642846303351</v>
+        <v>0.06315016804462398</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -1414,13 +1414,13 @@
         <v>25</v>
       </c>
       <c r="C63">
-        <v>0.0007966681746988872</v>
+        <v>0.0008701140895481975</v>
       </c>
       <c r="D63">
-        <v>0.0007903689940174771</v>
+        <v>0.0008183147699428881</v>
       </c>
       <c r="E63">
-        <v>0.3134689011169428</v>
+        <v>0.2876459281392774</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -1429,13 +1429,13 @@
         <v>26</v>
       </c>
       <c r="C64">
-        <v>0.03475081698811359</v>
+        <v>0.03272066963877188</v>
       </c>
       <c r="D64">
-        <v>0.02677616967509721</v>
+        <v>0.02711855165216932</v>
       </c>
       <c r="E64">
-        <v>0.1943470329636288</v>
+        <v>0.2275943934027006</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -1444,13 +1444,13 @@
         <v>27</v>
       </c>
       <c r="C65">
-        <v>-0.1281782785974296</v>
+        <v>-0.1409674049910742</v>
       </c>
       <c r="D65">
-        <v>0.07852236611018493</v>
+        <v>0.07684730827431988</v>
       </c>
       <c r="E65">
-        <v>0.1025996242968296</v>
+        <v>0.06659714374585926</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -1459,13 +1459,13 @@
         <v>28</v>
       </c>
       <c r="C66">
-        <v>0.009731397215447891</v>
+        <v>0.009640744575398191</v>
       </c>
       <c r="D66">
-        <v>0.004231987521186784</v>
+        <v>0.004175901396928083</v>
       </c>
       <c r="E66">
-        <v>0.02147734193191975</v>
+        <v>0.02096234849853482</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -1474,13 +1474,13 @@
         <v>29</v>
       </c>
       <c r="C67">
-        <v>0.2110598002789552</v>
+        <v>0.2188620217844745</v>
       </c>
       <c r="D67">
-        <v>0.07540914138098391</v>
+        <v>0.07532302008617478</v>
       </c>
       <c r="E67">
-        <v>0.005128300742430054</v>
+        <v>0.003664959835249084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>